<commit_message>
Clean URLs: name-based slugs for artists (/johann-vera), extensionless page URLs; keep artistaN internally via slug map; old artistaN.html kept as redirect stubs; cache-bust JS
</commit_message>
<xml_diff>
--- a/CRM_ToT.xlsx
+++ b/CRM_ToT.xlsx
@@ -751,7 +751,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>NEON16</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -765,26 +765,10 @@
           <t>EP.01 · 2025</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -905,26 +889,10 @@
           <t>EP.02 · 2025</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="inlineStr">
         <is>
@@ -1031,7 +999,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Intergroup Records</t>
+          <t>Independiente</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -1050,21 +1018,9 @@
           <t>370K</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1123,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>Warner Music Latina</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
@@ -1181,26 +1137,10 @@
           <t>EP.04 · 2025</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -1326,21 +1266,9 @@
           <t>25K</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>https://open.spotify.com/intl-es/artist/1YZcJWydWAbSpknMUKtD9m</t>
@@ -1465,26 +1393,10 @@
           <t>EP.06 · 2025</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -1591,7 +1503,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>777 Records</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -1610,21 +1522,9 @@
           <t>70K</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>https://open.spotify.com/intl-es/artist/6CHaM7DPIvAhLVOB5wNncN</t>
@@ -1731,7 +1631,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>Banchon Music</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
@@ -1745,26 +1645,10 @@
           <t>EP.08 · 2025</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -1885,26 +1769,10 @@
           <t>EP.09 · 2025</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -2011,7 +1879,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Emporio Records</t>
+          <t>Emporio Records / Warner Argentina</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
@@ -2025,26 +1893,14 @@
           <t>EP.10 · 2025</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
           <t>1.6M oyentes/mes</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>https://open.spotify.com/artist/2tsxhfhrjoqKy2okihHP0x</t>

</xml_diff>